<commit_message>
Schematic update and partial routing
</commit_message>
<xml_diff>
--- a/projects/LM5143_Buck/LM5143_BOM.xlsx
+++ b/projects/LM5143_Buck/LM5143_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\UWRT\MarsRoverElectricalKiCad\projects\LM5143_Buck\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4796AFC8-5DC9-4F86-83AE-D524F6B81D9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54266DE3-0BC9-4B88-9EC3-553AA017F7CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{49714629-2E5D-47B8-A555-D616FDA96D84}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="141">
   <si>
     <t>Capacitor In</t>
   </si>
@@ -455,7 +455,10 @@
     <t>*3 out of 10</t>
   </si>
   <si>
-    <t>*6 out of 5</t>
+    <t>*4 out of 5</t>
+  </si>
+  <si>
+    <t>*8 out of 100</t>
   </si>
 </sst>
 </file>
@@ -1775,14 +1778,14 @@
         <v>68</v>
       </c>
       <c r="C52">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="D52" s="1">
         <v>0.39</v>
       </c>
       <c r="E52" s="1">
         <f>IF(COUNT(C52:D52)=2,D52*C52*IF(ISNUMBER(SEARCH("lcsc", F52)), U$2, 1),"")</f>
-        <v>0.64116000000000006</v>
+        <v>0.4274400000000001</v>
       </c>
       <c r="F52" t="s">
         <v>67</v>
@@ -1853,20 +1856,20 @@
         <v>10</v>
       </c>
       <c r="C57">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="D57" s="1">
         <v>0.39</v>
       </c>
       <c r="E57" s="1">
         <f>IF(COUNT(C57:D57)=2,D57*C57*IF(ISNUMBER(SEARCH("lcsc", F57)), U$2, 1),"")</f>
-        <v>1.0686000000000001E-2</v>
+        <v>4.2744000000000004E-2</v>
       </c>
       <c r="F57" t="s">
         <v>135</v>
       </c>
       <c r="Q57" t="s">
-        <v>52</v>
+        <v>140</v>
       </c>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.35">
@@ -1994,7 +1997,7 @@
       </c>
       <c r="E66" s="1">
         <f>SUM(E2:E65)</f>
-        <v>100.083777</v>
+        <v>99.902114999999995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fully routed, no via stitching yet
</commit_message>
<xml_diff>
--- a/projects/LM5143_Buck/LM5143_BOM.xlsx
+++ b/projects/LM5143_Buck/LM5143_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\UWRT\MarsRoverElectricalKiCad\projects\LM5143_Buck\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54266DE3-0BC9-4B88-9EC3-553AA017F7CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02595036-1A80-474C-9C7F-4D3D47CE0D8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{49714629-2E5D-47B8-A555-D616FDA96D84}"/>
   </bookViews>
@@ -443,9 +443,6 @@
     <t>https://www.lcsc.com/product-detail/C189895.html</t>
   </si>
   <si>
-    <t>https://www.lcsc.com/product-detail/C109318.html</t>
-  </si>
-  <si>
     <t>RT0603FRE07390KL</t>
   </si>
   <si>
@@ -458,7 +455,10 @@
     <t>*4 out of 5</t>
   </si>
   <si>
-    <t>*8 out of 100</t>
+    <t>https://www.lcsc.com/product-detail/C861082.html</t>
+  </si>
+  <si>
+    <t>*8 out of 20</t>
   </si>
 </sst>
 </file>
@@ -1634,7 +1634,7 @@
         <v>43</v>
       </c>
       <c r="Q44" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.35">
@@ -1698,7 +1698,7 @@
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B48" t="s">
         <v>54</v>
@@ -1714,7 +1714,7 @@
         <v>1.4796000000000002E-2</v>
       </c>
       <c r="F48" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="Q48" t="s">
         <v>45</v>
@@ -1791,7 +1791,7 @@
         <v>67</v>
       </c>
       <c r="Q52" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.35">
@@ -1856,17 +1856,17 @@
         <v>10</v>
       </c>
       <c r="C57">
-        <v>0.08</v>
+        <v>0.4</v>
       </c>
       <c r="D57" s="1">
-        <v>0.39</v>
+        <v>0.94</v>
       </c>
       <c r="E57" s="1">
         <f>IF(COUNT(C57:D57)=2,D57*C57*IF(ISNUMBER(SEARCH("lcsc", F57)), U$2, 1),"")</f>
-        <v>4.2744000000000004E-2</v>
+        <v>0.51512000000000002</v>
       </c>
       <c r="F57" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="Q57" t="s">
         <v>140</v>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="E66" s="1">
         <f>SUM(E2:E65)</f>
-        <v>99.902114999999995</v>
+        <v>100.37449099999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>